<commit_message>
fix: delete outdated scripts and update imports
</commit_message>
<xml_diff>
--- a/experiments/04_lora_finetuning/report/best_models.xlsx
+++ b/experiments/04_lora_finetuning/report/best_models.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="best_models" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -562,7 +562,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>qwen_lora_7b_no_shots_2_epochs</t>
+          <t>qwen_lora_7b_zero_shot_2_epochs</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -571,7 +571,7 @@
       <c r="F1" s="3" t="n"/>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>gpt_4o_mini_few_shots</t>
+          <t>GPT-4o-mini</t>
         </is>
       </c>
       <c r="H1" s="2" t="n"/>

</xml_diff>